<commit_message>
feat(rental): standardize indemnity fee to ₹30 in Mumbai across engine, database, and docs
</commit_message>
<xml_diff>
--- a/Rental Final Table/LetzRyd_Rental_Master_Architecture_Complete.xlsx
+++ b/Rental Final Table/LetzRyd_Rental_Master_Architecture_Complete.xlsx
@@ -767,7 +767,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>public.rental_fee_rules — Daily indemnity insurance (Standard ₹30/day; Mumbai ₹0; Hyundai Xcent retired fleet ₹0; Waived partners ₹0). Net Daily Rent = Applied Rent + Applied Indemnity.</t>
+          <t>public.rental_fee_rules — Standardized daily indemnity insurance (Standard ₹30/day across all cities: Bangalore, Hyderabad, Mumbai; Hyundai Xcent retired fleet ₹0; Waived partners ₹0). Net Daily Rent = Applied Rent + Applied Indemnity.</t>
         </is>
       </c>
     </row>
@@ -806,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
@@ -815,7 +815,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="63" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
@@ -830,7 +830,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rules governing daily vehicle indemnity fees, model-specific waivers, and custom fee schedules (including Mumbai standard waiver).</t>
+          <t>Rules governing daily vehicle indemnity fees, model-specific waivers, and custom fee schedules.</t>
         </is>
       </c>
     </row>
@@ -843,7 +843,7 @@
       </c>
       <c r="B4" s="30" t="inlineStr">
         <is>
-          <t>fee_rule_id (SERIAL INT - Clean 1 to 7)</t>
+          <t>fee_rule_id (SERIAL INT - Clean 1 to 6)</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>1 row per fee policy or exemption rule (7 active rules)</t>
+          <t>1 row per fee policy or exemption rule (6 active rules)</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B8" s="30" t="inlineStr">
         <is>
-          <t>Resolves daily indemnity fee: Standard ₹30/day; Mumbai ₹0 (waiver); Xcent ₹0; Waived partners ₹0.</t>
+          <t>Resolves daily indemnity fee: Standard ₹30/day across all cities (Bangalore, Hyderabad, Mumbai); Xcent ₹0; Waived partners ₹0.</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Standard daily indemnity across all cities</t>
+          <t>Standard daily indemnity across all cities (Bangalore, Hyderabad, Mumbai)</t>
         </is>
       </c>
       <c r="H11" s="33" t="n">
@@ -1162,43 +1162,6 @@
         <v>46023</v>
       </c>
       <c r="I16" s="34" t="n">
-        <v>2958465</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="37" t="n">
-        <v>7</v>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Mumbai</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="31" t="b">
-        <v>1</v>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>Mumbai standard indemnity waiver (fee included in base rent)</t>
-        </is>
-      </c>
-      <c r="H17" s="33" t="n">
-        <v>46023</v>
-      </c>
-      <c r="I17" s="33" t="n">
         <v>2958465</v>
       </c>
     </row>
@@ -19865,7 +19828,7 @@
     <col width="65" customWidth="1" min="6" max="6"/>
     <col width="65" customWidth="1" min="7" max="7"/>
     <col width="65" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
     <col width="65" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -20491,8 +20454,8 @@
       <c r="G14" s="24" t="inlineStr">
         <is>
           <t>1. Calculates total weekly Uber trips.
-2. Matches into 6 discrete trip milestone tiers.
-3. Applies net rent (In Mumbai, base rent includes indemnity; standard fee is ₹0).</t>
+2. Matches into 6 discrete trip milestone tiers in rental_rate_slabs.
+3. Adds standard ₹30/day indemnity fee from rental_fee_rules.</t>
         </is>
       </c>
       <c r="H14" s="22" t="inlineStr">
@@ -20507,12 +20470,12 @@
       </c>
       <c r="I14" s="24" t="inlineStr">
         <is>
-          <t>₹0.00/day (Built into base)</t>
+          <t>₹30.00/day</t>
         </is>
       </c>
       <c r="J14" s="22" t="inlineStr">
         <is>
-          <t>Mumbai driver reaches 112 trips in the week. He enters the 110-124 slab (₹569/day). For 7 billable days, Total Rent = 7 × ₹569 = ₹3,983.</t>
+          <t>Mumbai driver reaches 112 trips in the week. He enters the 110-124 slab (₹569/day). Net rent = ₹569 + ₹30 = ₹599/day. For 7 billable days, Total Rent = 7 × ₹599 = ₹4,193.</t>
         </is>
       </c>
     </row>
@@ -20550,7 +20513,7 @@
       <c r="G15" s="21" t="inlineStr">
         <is>
           <t>1. Applies standard base rent of ₹1,100/day.
-2. Adds ₹30/day indemnity fee.
+2. Adds standard ₹30/day indemnity fee.
 3. Total net daily rent = ₹1,130/day.</t>
         </is>
       </c>
@@ -20598,28 +20561,28 @@
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
-          <t>Fixed-rate contract permitting dual-application driving.</t>
+          <t>Fixed-rate contract permitting dual-application driving with full company insurance cover.</t>
         </is>
       </c>
       <c r="G16" s="24" t="inlineStr">
         <is>
           <t>1. Applies flat rate ₹1,050/day.
-2. Fee is ₹0/day.</t>
+2. Adds standard ₹30/day indemnity fee.</t>
         </is>
       </c>
       <c r="H16" s="22" t="inlineStr">
         <is>
-          <t>• Flat ₹1,050/day</t>
+          <t>• Flat ₹1,050/day base rent</t>
         </is>
       </c>
       <c r="I16" s="24" t="inlineStr">
         <is>
-          <t>₹0.00/day</t>
+          <t>₹30.00/day</t>
         </is>
       </c>
       <c r="J16" s="22" t="inlineStr">
         <is>
-          <t>Driver operating across both platforms is billed 7 × ₹1,050 = ₹7,350.</t>
+          <t>Driver operating across both platforms is billed 7 × (1,050 + 30) = ₹7,560.</t>
         </is>
       </c>
     </row>
@@ -20657,24 +20620,24 @@
       <c r="G17" s="21" t="inlineStr">
         <is>
           <t>1. Fetches model baseline from rental_model_baselines.
-2. Applies city baseline rate.</t>
+2. Adds standard ₹30/day indemnity fee.</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>• WagonR: ₹970/day
-• Dzire / Aura: ₹1,100/day
-• Tigor EV: ₹1,300/day</t>
+          <t>• WagonR: ₹970 + ₹30 = ₹1,000/day
+• Dzire / Aura: ₹1,100 + ₹30 = ₹1,130/day
+• Tigor EV: ₹1,300 + ₹30 = ₹1,330/day</t>
         </is>
       </c>
       <c r="I17" s="21" t="inlineStr">
         <is>
-          <t>₹0.00/day</t>
+          <t>₹30.00/day</t>
         </is>
       </c>
       <c r="J17" s="19" t="inlineStr">
         <is>
-          <t>Mumbai WagonR with 0 trips is billed baseline rate: 7 × ₹970 = ₹6,790.</t>
+          <t>Mumbai WagonR with 0 trips is billed baseline rate: 7 × (970 + 30) = ₹7,000.</t>
         </is>
       </c>
     </row>
@@ -21791,7 +21754,7 @@
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
-          <t>Flat ₹1,050/day (Indemnity ₹0)</t>
+          <t>Flat ₹1,050/day + ₹30 fee = ₹1,080/day</t>
         </is>
       </c>
       <c r="H20" s="12" t="inlineStr">
@@ -21891,7 +21854,7 @@
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
-          <t>WagonR: ₹970, Dzire: ₹1,100, Tigor EV: ₹1,300</t>
+          <t>WagonR: ₹970, Dzire: ₹1,100, Tigor EV: ₹1,300 (+ ₹30 fee)</t>
         </is>
       </c>
       <c r="H22" s="12" t="inlineStr">
@@ -21941,7 +21904,7 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>WagonR 6 Tiers: ₹970 to ₹339/day (Indemnity ₹0)</t>
+          <t>WagonR 6 Tiers: ₹970 to ₹339/day + ₹30 fee</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">

</xml_diff>

<commit_message>
docs(rental): align Bangalore Master Individual slabs and statement walkthrough with rental_rate_slabs
</commit_message>
<xml_diff>
--- a/Rental Final Table/LetzRyd_Rental_Master_Architecture_Complete.xlsx
+++ b/Rental Final Table/LetzRyd_Rental_Master_Architecture_Complete.xlsx
@@ -19940,11 +19940,10 @@
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>• 0 - 54 trips: ₹929/day
-• 55 - 64 trips: ₹899/day
-• 65 - 74 trips: ₹879/day
-• 75 - 89 trips: ₹869/day
-• 90+ trips: ₹799/day
+          <t>• 0 - 89 trips: ₹929/day
+• 90 - 109 trips: ₹665/day
+• 110 - 129 trips: ₹525/day
+• 130+ trips: ₹400/day
 • Ola trips &gt;= 1: Flat ₹1,050/day</t>
         </is>
       </c>
@@ -19955,8 +19954,8 @@
       </c>
       <c r="J5" s="19" t="inlineStr">
         <is>
-          <t>Driver A completes 68 Uber trips and 0 Ola trips in the week. He lands in the 65-74 tier (₹879/day). For 7 active billable days, Rent = 7 × (879 + 30) = ₹6,363.
-If Driver A did 67 Uber trips and 1 Ola trip, he is penalized: Rent = 7 × (1050 + 30) = ₹7,560.</t>
+          <t>Driver A completes 102 Uber trips and 0 Ola trips in the week. He lands in the 90-109 tier (₹665/day). For 7 active billable days, Rent = 7 × (665 + 30) = ₹4,865.
+If Driver A did 101 Uber trips and 1 Ola trip, he is penalized: Rent = 7 × (1,050 + 30) = ₹7,560.</t>
         </is>
       </c>
     </row>
@@ -20776,7 +20775,7 @@
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>Uber Completed Trips = 68, Ola Completed Trips = 0, Total Trips = 68</t>
+          <t>Uber Completed Trips = 102, Ola Completed Trips = 0, Total Trips = 102</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -20786,7 +20785,7 @@
       </c>
       <c r="G6" s="22" t="inlineStr">
         <is>
-          <t>Weekly Trips = 68 (Ola = 0)</t>
+          <t>Weekly Trips = 102 (Ola = 0)</t>
         </is>
       </c>
     </row>
@@ -20882,22 +20881,22 @@
       </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
-          <t>city = 'Bangalore', customer_type = 'Individual', vehicle_model = 'WagonR', trips = 68, plan_id = 'BLR_MASTER_IND'</t>
+          <t>city = 'Bangalore', customer_type = 'Individual', vehicle_model = 'WagonR', trips = 102, plan_id = 'BLR_MASTER_IND'</t>
         </is>
       </c>
       <c r="E9" s="21" t="inlineStr">
         <is>
-          <t>Trip Tier: 65 to 74 trips -&gt; base_daily_rent = ₹879.00/day</t>
+          <t>Trip Tier: 90 to 109 trips -&gt; base_daily_rent = ₹665.00/day</t>
         </is>
       </c>
       <c r="F9" s="21" t="inlineStr">
         <is>
-          <t>Under BLR_MASTER_IND, because Ola trips = 0, no multi-app penalty is triggered. Driver earns Tier 3 discount (₹879 vs ₹929 base).</t>
+          <t>Under BLR_MASTER_IND, because Ola trips = 0, no multi-app penalty is triggered. Driver earns Tier 2 discount (₹665 vs ₹929 base).</t>
         </is>
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Base Daily Rent = ₹879.00/day</t>
+          <t>Base Daily Rent = ₹665.00/day</t>
         </is>
       </c>
     </row>
@@ -20961,17 +20960,17 @@
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>Row inserted: applied_rent = 879.00, indemnity = 30.00, net_rent = 909.00</t>
+          <t>Row inserted: applied_rent = 665.00, indemnity = 30.00, net_rent = 695.00</t>
         </is>
       </c>
       <c r="F11" s="21" t="inlineStr">
         <is>
-          <t>Committed into daily rent log with audit rule: 'Priority 3: Dynamic Slab (BLR_MASTER_IND: 65-74)'. Tri-grain protects against handover collisions.</t>
+          <t>Committed into daily rent log with audit rule: 'Priority 3: Dynamic Slab (BLR_MASTER_IND: 90-109)'. Tri-grain protects against handover collisions.</t>
         </is>
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Net Daily Rent = ₹909.00/day</t>
+          <t>Net Daily Rent = ₹695.00/day</t>
         </is>
       </c>
     </row>
@@ -20998,7 +20997,7 @@
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>Daily ledger row updated with lease_rental = ₹879.00, indemnity = ₹30.00</t>
+          <t>Daily ledger row updated with lease_rental = ₹665.00, indemnity = ₹30.00</t>
         </is>
       </c>
       <c r="F12" s="24" t="inlineStr">
@@ -21035,7 +21034,7 @@
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>Weekly Lease Rental = 7 × ₹879 = ₹6,153.00 | Weekly Indemnity = 7 × ₹30 = ₹210.00</t>
+          <t>Weekly Lease Rental = 7 × ₹665 = ₹4,655.00 | Weekly Indemnity = 7 × ₹30 = ₹210.00</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -21045,7 +21044,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>TOTAL WEEKLY RENT = ₹6,363.00</t>
+          <t>TOTAL WEEKLY RENT = ₹4,865.00</t>
         </is>
       </c>
     </row>

</xml_diff>